<commit_message>
Competitor analysis against the MVP; Design and Features notes filled in
- docs/ANALISI_COMPETITOR.md: summary of the research, what only MyFinancePlace does, what is missing,
  decisions to take (double-entry, licence, web or desktop, Italian tax)
- Analisi Funzionalita vs MVP.xlsx: 37 features × 12 apps with a computed score, corrections to the two
  strategy workbooks, missing competitors (Sure, PocketSmith, Lunch Money…), analyses to add, sources
- Analisi Strategica.xlsx: «Design and Features Notes» filled for all 45 apps (score + notes); only that
  sheet's XML was edited, so the chart, comments and tables are untouched

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Strategy and Business/Analisi Strategica.xlsx
+++ b/docs/Strategy and Business/Analisi Strategica.xlsx
@@ -2858,7 +2858,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3063,6 +3063,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -18756,316 +18759,808 @@
       <c r="A5" s="68" t="s">
         <v>423</v>
       </c>
-      <c r="B5" s="69"/>
-      <c r="C5" s="69"/>
+      <c r="B5" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 7/10
+• Linguaggio visivo ispirato a Monarch: KPI in card, grafici Plotly, tema chiaro/scuro, menu laterale comprimibile, uso da telefono
+• Interfaccia completa in italiano e inglese
+• Deboli: nessun onboarding guidato, niente scorciatoie da tastiera né annulla, tante voci nel menu (serve una gerarchia più chiara)
+• Da fare: tabella Riepilogo e Sankey per raccontare i dati; un tour iniziale come quello di Actual 26.9</t>
+        </is>
+      </c>
+      <c r="C5" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Transazioni con segno, tag da un elenco, regole scritte o imparate, classificazione con AI locale
+• Import di 8 banche italiane + formato generico (Excel, CSV, PDF, Word, ODF, RTF), OCR/AI con conferma, controllo duplicati
+• Dashboard annuale, report, budget con avvisi, obiettivi, previsione con 6 metodi
+• SP/CE/CF, patrimonio netto, portafoglio, debiti, assicurazioni, documenti, snapshot, più valute, backup .zip
+• Mancano: transazioni suddivise, riporto del budget, Sankey, OFX/CAMT, partita doppia vera, licenza</t>
+        </is>
+      </c>
     </row>
     <row r="6" spans="1:5" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="68" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="69"/>
-      <c r="C6" s="69"/>
+      <c r="B6" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• App mobile curata: card colorate e grafici ricchi; web app completa
+• Molte funzioni dietro il premium, la navigazione a volte è dispersiva
+• Da prendere: dashboard componibile a widget</t>
+        </is>
+      </c>
+      <c r="C6" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• Collegamento alle banche UE (anche italiane) via Salt Edge, più conti e valute, budget, pagamenti pianificati suggeriti, report, conti condivisi
+• Niente partita doppia né SP/CE
+• Rispetto a MFP: vince su sync e mobile, perde su import da file, rendiconti e privacy</t>
+        </is>
+      </c>
     </row>
     <row r="7" spans="1:5" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="68" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="69"/>
-      <c r="C7" s="69"/>
+      <c r="B7" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Molto visuale: colori per categoria, grafici semplici, onboarding leggero; pensata per il telefono
+• Da prendere: portafogli separati e condivisi con icone chiare</t>
+        </is>
+      </c>
+      <c r="C7" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 5/10
+• Budget, portafogli condivisi, collegamento banche, categorie, più valute, grafici delle spese
+• Niente investimenti, rendiconti né previsione
+• Rispetto a MFP: punta su coppie e famiglie, fuori dal nostro perimetro</t>
+        </is>
+      </c>
     </row>
     <row r="8" spans="1:5" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="68" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="69"/>
-      <c r="C8" s="69"/>
+      <c r="B8" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• Interfaccia funzionale, stile Android classico; sviluppata in Italia
+• Da verificare aprendo l'app</t>
+        </is>
+      </c>
+      <c r="C8" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 5/10
+• Movimenti, categorie e sottocategorie flessibili, budget, promemoria, più conti, sync opzionale
+• Rispetto a MFP: concorrente italiano semplice, senza rendiconti né import di estratti conto</t>
+        </is>
+      </c>
     </row>
     <row r="9" spans="1:5" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="68" t="s">
         <v>70</v>
       </c>
-      <c r="B9" s="69"/>
-      <c r="C9" s="69"/>
+      <c r="B9" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Densa ma chiara: schede giorno / calendario / mese / totale, entrate in blu e uscite in rosso
+• La vista calendario è la più apprezzata
+• Da prendere: calendario con i totali giornalieri</t>
+        </is>
+      </c>
+      <c r="C9" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• Conti attività/passività con partita doppia automatica (conto ↔ categoria), budget settimanali/mensili/annuali, statistiche, ricorrenti, gestione da PC via Wi-Fi, export Excel
+• Niente investimenti seri né SP/CE
+• Rispetto a MFP: più forte sull'inserimento rapido da telefono</t>
+        </is>
+      </c>
     </row>
     <row r="10" spans="1:5" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="68" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="69"/>
-      <c r="C10" s="69"/>
+      <c r="B10" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Inserimento a icone rapidissimo: una torta con le categorie intorno, due tocchi per registrare
+• Da prendere: velocità di inserimento</t>
+        </is>
+      </c>
+      <c r="C10" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 3/10
+• Entrate/uscite, categorie, budget semplice, sync, più valute
+• Un registro di spese, non un gestionale</t>
+        </is>
+      </c>
     </row>
     <row r="11" spans="1:5" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="68" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="69"/>
-      <c r="C11" s="69"/>
+      <c r="B11" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Interfaccia costruita attorno al metodo: colore di stato (verde / giallo / rosso) su ogni categoria
+• Onboarding ed educazione finanziaria eccellenti; curva di apprendimento alta
+• Da prendere: stato della categoria leggibile a colpo d'occhio</t>
+        </is>
+      </c>
+      <c r="C11" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• Budget a base zero, Targets settimanali/mensili/annuali, Age of Money, Reflect (patrimonio, spese, entrate), collegamento banche USA e parte dell'UE, pianificatore prestiti, condivisione
+• Niente investimenti, una sola valuta per budget
+• Rispetto a MFP: metodo forte, nessun rendiconto</t>
+        </is>
+      </c>
     </row>
     <row r="12" spans="1:5" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="68" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="69"/>
-      <c r="C12" s="69"/>
+      <c r="B12" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• Semplice e guidata dal metodo Ramsey; pochi grafici</t>
+        </is>
+      </c>
+      <c r="C12" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 3/10
+• Budget a base zero, tracciamento spese, obiettivi; collegamento banche solo premium; solo USA</t>
+        </is>
+      </c>
     </row>
     <row r="13" spans="1:5" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="69"/>
-      <c r="C13" s="69"/>
+      <c r="B13" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• La metafora delle buste è ben visibile; interfaccia un po' datata</t>
+        </is>
+      </c>
+      <c r="C13" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 4/10
+• Buste digitali, budget, sync tra dispositivi, debiti; inserimento solo manuale</t>
+        </is>
+      </c>
     </row>
     <row r="14" spans="1:5" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="68" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="69"/>
-      <c r="C14" s="69"/>
+      <c r="B14" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• Un numero al centro («In My Pocket»); per il resto un'app standard
+• Da prendere: il numero «quanto posso ancora spendere» (con spese fisse / variabili)</t>
+        </is>
+      </c>
+      <c r="C14" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 4/10
+• Saldo spendibile, budget automatico, bollette, categorie, risparmio; solo USA</t>
+        </is>
+      </c>
     </row>
     <row r="15" spans="1:5" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="68" t="s">
         <v>147</v>
       </c>
-      <c r="B15" s="69"/>
-      <c r="C15" s="69"/>
+      <c r="B15" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• Minimale e pulita, pochi schermi</t>
+        </is>
+      </c>
+      <c r="C15" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 3/10
+• Entrate/uscite, budget, categorie, più valute, export</t>
+        </is>
+      </c>
     </row>
     <row r="16" spans="1:5" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="68" t="s">
         <v>152</v>
       </c>
-      <c r="B16" s="69"/>
-      <c r="C16" s="69"/>
+      <c r="B16" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• Essenziale, solo Android; da verificare aprendo l'app</t>
+        </is>
+      </c>
+      <c r="C16" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 3/10
+• Budget familiare mensile, categorie, report, promemoria</t>
+        </is>
+      </c>
     </row>
     <row r="17" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="68" t="s">
         <v>158</v>
       </c>
-      <c r="B17" s="69"/>
-      <c r="C17" s="69"/>
+      <c r="B17" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 5/10
+• Inserimento rapido, anche a voce secondo la mappatura; da verificare
+• Da prendere: inserimento in linguaggio naturale («pizza 12 euro») con l'AI già presente in MFP</t>
+        </is>
+      </c>
+      <c r="C17" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 2/10
+• Tracciamento spese, categorie, statistiche</t>
+        </is>
+      </c>
     </row>
     <row r="18" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="68" t="s">
         <v>163</v>
       </c>
-      <c r="B18" s="69"/>
-      <c r="C18" s="69"/>
+      <c r="B18" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 5/10
+• App Windows semplice con registro a tabella; da verificare</t>
+        </is>
+      </c>
+      <c r="C18" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 2/10
+• Registro entrate/uscite, budget, grafici</t>
+        </is>
+      </c>
     </row>
     <row r="19" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="68" t="s">
         <v>168</v>
       </c>
-      <c r="B19" s="69"/>
-      <c r="C19" s="69"/>
+      <c r="B19" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 4/10
+• Interfaccia Windows spartana; da verificare</t>
+        </is>
+      </c>
+      <c r="C19" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 2/10
+• Budget per categorie, report di base</t>
+        </is>
+      </c>
     </row>
     <row r="20" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="68" t="s">
         <v>172</v>
       </c>
-      <c r="B20" s="69"/>
-      <c r="C20" s="69"/>
+      <c r="B20" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• Il calendario è l'interfaccia principale
+• Da prendere: heatmap delle spese giornaliere</t>
+        </is>
+      </c>
+      <c r="C20" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 3/10
+• Vista a calendario, entrate/uscite, budget mensile</t>
+        </is>
+      </c>
     </row>
     <row r="21" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="68" t="s">
         <v>176</v>
       </c>
-      <c r="B21" s="69"/>
-      <c r="C21" s="69"/>
+      <c r="B21" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Curata e coerente tra iOS, macOS e Windows; scadenzario molto visivo</t>
+        </is>
+      </c>
+      <c r="C21" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 7/10
+• Budget, bollette e scadenze, conti, collegamento banche, report, più valute, più dispositivi; investimenti limitati</t>
+        </is>
+      </c>
     </row>
     <row r="22" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="68" t="s">
         <v>185</v>
       </c>
-      <c r="B22" s="69"/>
-      <c r="C22" s="69"/>
+      <c r="B22" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• App Windows essenziale; da verificare</t>
+        </is>
+      </c>
+      <c r="C22" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 3/10
+• Budget, spese, obiettivi, grafici</t>
+        </is>
+      </c>
     </row>
     <row r="23" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="68" t="s">
         <v>188</v>
       </c>
-      <c r="B23" s="69"/>
-      <c r="C23" s="69"/>
+      <c r="B23" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 4/10
+• Interfaccia Windows spartana; da verificare</t>
+        </is>
+      </c>
+      <c r="C23" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 2/10
+• Analisi e revisione del budget, categorie, report</t>
+        </is>
+      </c>
     </row>
     <row r="24" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="68" t="s">
         <v>268</v>
       </c>
-      <c r="B24" s="69"/>
-      <c r="C24" s="69"/>
+      <c r="B24" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• Molto completa ma densa, interfaccia desktop di vecchia scuola; Simplifi è la versione moderna</t>
+        </is>
+      </c>
+      <c r="C24" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Budget, conti e investimenti (Classic), bollette, report fiscali, prestiti, file locale + cloud; solo USA
+• Rispetto a MFP: il riferimento storico per ampiezza, niente Italia</t>
+        </is>
+      </c>
     </row>
     <row r="25" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="68" t="s">
         <v>278</v>
       </c>
-      <c r="B25" s="69"/>
-      <c r="C25" s="69"/>
+      <c r="B25" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 10/10
+• Il riferimento del mercato: dashboard a card, Sankey, grafici puliti, tipografia e colori sobri; web e mobile allineati
+• È l'ispirazione dichiarata della UI di MFP</t>
+        </is>
+      </c>
+      <c r="C25" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 9/10
+• Collegamento conti, budget Flex (fisse / non mensili / variabili) o per categoria con riporto, Cash Flow con Sankey e tasso di risparmio, previsione del saldo, obiettivi, ricorrenti rilevati, regole, tag, split, investimenti, assistente AI, collaborazione
+• Rispetto a MFP: niente rendiconti, solo USA/Canada, solo cloud</t>
+        </is>
+      </c>
     </row>
     <row r="26" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="68" t="s">
         <v>20</v>
       </c>
-      <c r="B26" s="69"/>
-      <c r="C26" s="69"/>
+      <c r="B26" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• App di trading semplice e quasi ludica</t>
+        </is>
+      </c>
+      <c r="C26" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 3/10
+• Non è un PFM: trading di azioni, ETF, opzioni e cripto, gestione della liquidità; nessun budget</t>
+        </is>
+      </c>
     </row>
     <row r="27" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="B27" s="69"/>
-      <c r="C27" s="69"/>
+      <c r="B27" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Onboarding semplicissimo, grafici essenziali</t>
+        </is>
+      </c>
+      <c r="C27" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 3/10
+• Arrotondamenti investiti, portafogli gestiti, pensione; nessun budget</t>
+        </is>
+      </c>
     </row>
     <row r="28" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="B28" s="69"/>
-      <c r="C28" s="69"/>
+      <c r="B28" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Pulita, organizzata per obiettivi</t>
+        </is>
+      </c>
+      <c r="C28" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 4/10
+• Robo-advisor, portafogli automatici, obiettivi, pensione, tax-loss harvesting</t>
+        </is>
+      </c>
     </row>
     <row r="29" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="68" t="s">
         <v>23</v>
       </c>
-      <c r="B29" s="69"/>
-      <c r="C29" s="69"/>
+      <c r="B29" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Pulita, con simulazioni interattive del piano</t>
+        </is>
+      </c>
+      <c r="C29" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 4/10
+• Robo-advisor, pianificazione, conto di liquidità, tax-loss harvesting</t>
+        </is>
+      </c>
     </row>
     <row r="30" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="68" t="s">
         <v>214</v>
       </c>
-      <c r="B30" s="69"/>
-      <c r="C30" s="69"/>
+      <c r="B30" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Social: feed della community, grafici di portafoglio moderni
+• Da prendere: vista dividendi e allocazione per il modulo Portafoglio</t>
+        </is>
+      </c>
+      <c r="C30" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 5/10
+• Portafoglio di azioni, ETF e cripto collegato ai broker, dividendi, analisi, community; nessun budget</t>
+        </is>
+      </c>
     </row>
     <row r="31" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="68" t="s">
         <v>224</v>
       </c>
-      <c r="B31" s="69"/>
-      <c r="C31" s="69"/>
+      <c r="B31" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Dashboard del patrimonio chiara; l'app spinge verso la consulenza a pagamento</t>
+        </is>
+      </c>
+      <c r="C31" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• Collegamento conti, patrimonio netto, fee analyzer, pianificazione pensione, budget di base; solo USA</t>
+        </is>
+      </c>
     </row>
     <row r="32" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="68" t="s">
         <v>234</v>
       </c>
-      <c r="B32" s="69"/>
-      <c r="C32" s="69"/>
+      <c r="B32" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• Web funzionale, orientata ai report</t>
+        </is>
+      </c>
+      <c r="C32" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 5/10
+• Performance, dividendi, report fiscali su plus/minusvalenze, più valute, import dai broker
+• Da prendere: report fiscale sugli investimenti</t>
+        </is>
+      </c>
     </row>
     <row r="33" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="68" t="s">
         <v>244</v>
       </c>
-      <c r="B33" s="69"/>
-      <c r="C33" s="69"/>
+      <c r="B33" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• Ricca di dati, densa</t>
+        </is>
+      </c>
+      <c r="C33" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 5/10
+• Ricerca e rating, X-Ray del portafoglio, screener, watchlist</t>
+        </is>
+      </c>
     </row>
     <row r="34" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="68" t="s">
         <v>252</v>
       </c>
-      <c r="B34" s="69"/>
-      <c r="C34" s="69"/>
+      <c r="B34" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Un «foglio di calcolo» elegante: righe di attività modificabili al volo, minimalista
+• Da prendere: modifica inline del valore di un'attività</t>
+        </is>
+      </c>
+      <c r="C34" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• Patrimonio multi-asset (cripto, immobili, metalli), proiezioni, beneficiari; nessun budget</t>
+        </is>
+      </c>
     </row>
     <row r="35" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="68" t="s">
         <v>261</v>
       </c>
-      <c r="B35" s="69"/>
-      <c r="C35" s="69"/>
+      <c r="B35" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• Calcolatore web semplice, in italiano</t>
+        </is>
+      </c>
+      <c r="C35" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 2/10
+• Capitale FIRE, tasso di prelievo, anni all'indipendenza
+• Da prendere: proiezione FIRE nella pagina Previsioni</t>
+        </is>
+      </c>
     </row>
     <row r="36" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="68" t="s">
         <v>41</v>
       </c>
-      <c r="B36" s="69"/>
-      <c r="C36" s="69"/>
+      <c r="B36" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• App bancaria di riferimento per design: card, animazioni, statistiche immediate</t>
+        </is>
+      </c>
+      <c r="C36" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 4/10
+• Conto multivaluta, budget per categoria, salvadanai con arrotondamento, investimenti, cripto; vede solo i conti Revolut</t>
+        </is>
+      </c>
     </row>
     <row r="37" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="68" t="s">
         <v>44</v>
       </c>
-      <c r="B37" s="69"/>
-      <c r="C37" s="69"/>
+      <c r="B37" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Minimalista, statistiche mensili chiare</t>
+        </is>
+      </c>
+      <c r="C37" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 3/10
+• Spaces (sotto-conti) con regole di trasferimento, statistiche, notifiche</t>
+        </is>
+      </c>
     </row>
     <row r="38" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="68" t="s">
         <v>47</v>
       </c>
-      <c r="B38" s="69"/>
-      <c r="C38" s="69"/>
+      <c r="B38" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Moderna, pensata per i più giovani</t>
+        </is>
+      </c>
+      <c r="C38" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 4/10
+• Obiettivi di risparmio, aggregatore PSD2 per vedere altre banche, cashback, investimenti di base</t>
+        </is>
+      </c>
     </row>
     <row r="39" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="68" t="s">
         <v>50</v>
       </c>
-      <c r="B39" s="69"/>
-      <c r="C39" s="69"/>
+      <c r="B39" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• App XME funzionale ma carica di servizi bancari</t>
+        </is>
+      </c>
+      <c r="C39" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 4/10
+• Categorizzazione automatica, Salvadanaio, limiti di spesa; solo per i clienti</t>
+        </is>
+      </c>
     </row>
     <row r="40" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="B40" s="69"/>
-      <c r="C40" s="69"/>
+      <c r="B40" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Business moderna e pulita</t>
+        </is>
+      </c>
+      <c r="C40" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 5/10
+• Budget per team e progetti, carte con limiti, gestione spese, fatturazione; non è un concorrente</t>
+        </is>
+      </c>
     </row>
     <row r="41" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="68" t="s">
         <v>55</v>
       </c>
-      <c r="B41" s="69"/>
-      <c r="C41" s="69"/>
+      <c r="B41" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Business moderna, pensata per le partite IVA</t>
+        </is>
+      </c>
+      <c r="C41" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 5/10
+• Flussi di cassa, accantonamento automatico per le tasse, F24
+• Da prendere: accantonamento delle tasse sui redditi da freelance</t>
+        </is>
+      </c>
     </row>
     <row r="42" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="68" t="s">
         <v>193</v>
       </c>
-      <c r="B42" s="69"/>
-      <c r="C42" s="69"/>
+      <c r="B42" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Moderna e veloce, si usa bene da tastiera; tema chiaro/scuro e temi personalizzati; tour iniziale (26.9.0)
+• Da prendere: inserimento da tastiera e annulla/ripeti</t>
+        </is>
+      </c>
+      <c r="C42" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 7/10
+• Budget a buste, regole, transazioni programmate con rilevamento dei ricorrenti, split, riconciliazione, report personalizzabili, Sankey e Age of Money (sperimentali), import OFX/QIF/CAMT/CSV, sync GoCardless/SimpleFIN, API, un file SQLite per budget
+• Niente investimenti né rendiconti</t>
+        </is>
+      </c>
     </row>
     <row r="43" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="68" t="s">
         <v>194</v>
       </c>
-      <c r="B43" s="69"/>
-      <c r="C43" s="69"/>
+      <c r="B43" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Minimalista; vista del patrimonio con attività/passività molto pulita
+• Da prendere: la pagina del patrimonio</t>
+        </is>
+      </c>
+      <c r="C43" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 7/10
+• Oggi continua come Sure: patrimonio, investimenti con benchmark, regole, budget con riporto e obiettivi (Sure 0.7.4, settembre 2026), chat AI, più valute, self-hosted
+• Maybe è archiviato, Sure è attivo</t>
+        </is>
+      </c>
     </row>
     <row r="44" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="68" t="s">
         <v>296</v>
       </c>
-      <c r="B44" s="69"/>
-      <c r="C44" s="69"/>
+      <c r="B44" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• Desktop pulita (Tauri), pochi schermi</t>
+        </is>
+      </c>
+      <c r="C44" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 5/10
+• Conti e titoli, performance, allocazione, obiettivi, import CSV, dati in locale; nessun budget</t>
+        </is>
+      </c>
     </row>
     <row r="45" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="68" t="s">
         <v>307</v>
       </c>
-      <c r="B45" s="69"/>
-      <c r="C45" s="69"/>
+      <c r="B45" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 4/10
+• Registro contabile tradizionale, menu e finestre datati: respinge chi non è contabile</t>
+        </is>
+      </c>
+      <c r="C45" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 7/10
+• Partita doppia completa, piano dei conti, riconciliazione, scadenzario, investimenti con quotazioni, report SP/CE/CF, budget, fatturazione di base, file locale
+• Rispetto a MFP: la profondità contabile da raggiungere</t>
+        </is>
+      </c>
     </row>
     <row r="46" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="68" t="s">
         <v>324</v>
       </c>
-      <c r="B46" s="69"/>
-      <c r="C46" s="69"/>
+      <c r="B46" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 3/10
+• File di testo + interfaccia web Fava: chiara per chi programma, ostica per tutti gli altri</t>
+        </is>
+      </c>
+      <c r="C46" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• Partita doppia in testo semplice, query BQL, bilanci generati, più valute, versionabile in Git; import tramite script</t>
+        </is>
+      </c>
     </row>
     <row r="47" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="68" t="s">
         <v>337</v>
       </c>
-      <c r="B47" s="69"/>
-      <c r="C47" s="69"/>
+      <c r="B47" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• Web utilitaristica con molte pagine; migliorata nel 2026 (font, ordinamento delle liste)</t>
+        </is>
+      </c>
+      <c r="C47" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 7/10
+• Conti tipizzati, partita doppia interna, budget e auto-budget, salvadanai, bollette, ricorrenti, regole, tag, split, più valute, API REST, data importer (GoCardless, CAMT, CSV)</t>
+        </is>
+      </c>
     </row>
     <row r="48" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="68" t="s">
         <v>351</v>
       </c>
-      <c r="B48" s="69"/>
-      <c r="C48" s="69"/>
+      <c r="B48" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 4/10
+• Desktop KDE tradizionale</t>
+        </is>
+      </c>
+      <c r="C48" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 6/10
+• Partita doppia, investimenti, scadenzario, budget, report, online banking (OFX/HBCI)</t>
+        </is>
+      </c>
     </row>
     <row r="49" spans="1:3" s="66" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="68" t="s">
         <v>362</v>
       </c>
-      <c r="B49" s="69"/>
-      <c r="C49" s="69"/>
+      <c r="B49" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Nativa Mac/iOS e curata; la v10 (maggio 2026) aggiunge Organizer, registro a riga singola e scala dell'interfaccia</t>
+        </is>
+      </c>
+      <c r="C49" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voto 8/10
+• Partita doppia, budget a buste, transazioni programmate avanzate, investimenti (IRR, ROI), report entrate/uscite e patrimonio anche su iOS, archiviazione degli anni chiusi, sync; solo Apple, orientata agli USA</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>